<commit_message>
remove B-fac>40 water from protein-compound set
</commit_message>
<xml_diff>
--- a/SI/Supplementary Data S1/ncryst.xlsx
+++ b/SI/Supplementary Data S1/ncryst.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\GitHub\WatGNN\watgnn\SI\number_of_crystallographic_water\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\GitHub\WatGNN_SI\SI\Supplementary Data S1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3DB1DE4-3CA0-4309-B3D3-8C917BF212C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B645B3A-C81C-4182-B02D-E8CEB7064D8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2400" yWindow="1920" windowWidth="28800" windowHeight="11295" firstSheet="1" activeTab="5" xr2:uid="{EE483F5B-5A14-4BEB-82EA-32D6D02872BB}"/>
+    <workbookView xWindow="1200" yWindow="1425" windowWidth="23040" windowHeight="11295" firstSheet="2" activeTab="4" xr2:uid="{EE483F5B-5A14-4BEB-82EA-32D6D02872BB}"/>
   </bookViews>
   <sheets>
     <sheet name="ncryst_WatGNN_train" sheetId="2" r:id="rId1"/>
@@ -24874,11 +24874,11 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>7.7±5.5</t>
+    <t>1–22</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>1–29</t>
+    <t>5.9±4.5</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -114485,23 +114485,23 @@
         <v>8240</v>
       </c>
       <c r="C2">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="E2">
         <f>SUM(C2:C172)</f>
-        <v>1318</v>
+        <v>1003</v>
       </c>
       <c r="F2">
         <f>AVERAGE(C2:C172)</f>
-        <v>7.7076023391812862</v>
+        <v>5.8654970760233915</v>
       </c>
       <c r="G2">
         <f>_xlfn.STDEV.P(C2:C172)</f>
-        <v>5.4715532914167291</v>
+        <v>4.4629117712611821</v>
       </c>
       <c r="H2">
         <f>MEDIAN(C2:C172)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I2">
         <f>MIN(C2:C172)</f>
@@ -114509,7 +114509,7 @@
       </c>
       <c r="J2">
         <f>MAX(C2:C172)</f>
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -114520,7 +114520,7 @@
         <v>8239</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -114542,7 +114542,7 @@
         <v>8237</v>
       </c>
       <c r="C5">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -114553,7 +114553,7 @@
         <v>8236</v>
       </c>
       <c r="C6">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -114575,7 +114575,7 @@
         <v>8234</v>
       </c>
       <c r="C8">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -114586,7 +114586,7 @@
         <v>8233</v>
       </c>
       <c r="C9">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -114608,7 +114608,7 @@
         <v>8231</v>
       </c>
       <c r="C11">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -114630,7 +114630,7 @@
         <v>8229</v>
       </c>
       <c r="C13">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -114641,7 +114641,7 @@
         <v>8228</v>
       </c>
       <c r="C14">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -114652,7 +114652,7 @@
         <v>8227</v>
       </c>
       <c r="C15">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -114663,7 +114663,7 @@
         <v>8226</v>
       </c>
       <c r="C16">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -114707,7 +114707,7 @@
         <v>8222</v>
       </c>
       <c r="C20">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -114729,7 +114729,7 @@
         <v>8220</v>
       </c>
       <c r="C22">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -114740,7 +114740,7 @@
         <v>8219</v>
       </c>
       <c r="C23">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -114762,7 +114762,7 @@
         <v>8217</v>
       </c>
       <c r="C25">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -114773,7 +114773,7 @@
         <v>8216</v>
       </c>
       <c r="C26">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -114795,7 +114795,7 @@
         <v>8214</v>
       </c>
       <c r="C28">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -114817,7 +114817,7 @@
         <v>8212</v>
       </c>
       <c r="C30">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -114839,7 +114839,7 @@
         <v>8210</v>
       </c>
       <c r="C32">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -114850,7 +114850,7 @@
         <v>8209</v>
       </c>
       <c r="C33">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -114861,7 +114861,7 @@
         <v>8208</v>
       </c>
       <c r="C34">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -114883,7 +114883,7 @@
         <v>8206</v>
       </c>
       <c r="C36">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -114905,7 +114905,7 @@
         <v>8204</v>
       </c>
       <c r="C38">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -114927,7 +114927,7 @@
         <v>8202</v>
       </c>
       <c r="C40">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -114938,7 +114938,7 @@
         <v>8201</v>
       </c>
       <c r="C41">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -114982,7 +114982,7 @@
         <v>8197</v>
       </c>
       <c r="C45">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -114993,7 +114993,7 @@
         <v>8196</v>
       </c>
       <c r="C46">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -115004,7 +115004,7 @@
         <v>8195</v>
       </c>
       <c r="C47">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="48" spans="1:3">
@@ -115059,7 +115059,7 @@
         <v>8190</v>
       </c>
       <c r="C52">
-        <v>14</v>
+        <v>5</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -115070,7 +115070,7 @@
         <v>8189</v>
       </c>
       <c r="C53">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -115092,7 +115092,7 @@
         <v>8187</v>
       </c>
       <c r="C55">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -115103,7 +115103,7 @@
         <v>8186</v>
       </c>
       <c r="C56">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -115125,7 +115125,7 @@
         <v>8184</v>
       </c>
       <c r="C58">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -115136,7 +115136,7 @@
         <v>8183</v>
       </c>
       <c r="C59">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -115147,7 +115147,7 @@
         <v>8182</v>
       </c>
       <c r="C60">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -115158,7 +115158,7 @@
         <v>8181</v>
       </c>
       <c r="C61">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -115169,7 +115169,7 @@
         <v>8180</v>
       </c>
       <c r="C62">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -115180,7 +115180,7 @@
         <v>8179</v>
       </c>
       <c r="C63">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -115257,7 +115257,7 @@
         <v>8172</v>
       </c>
       <c r="C70">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -115268,7 +115268,7 @@
         <v>8171</v>
       </c>
       <c r="C71">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="72" spans="1:3">
@@ -115279,7 +115279,7 @@
         <v>8170</v>
       </c>
       <c r="C72">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -115290,7 +115290,7 @@
         <v>8169</v>
       </c>
       <c r="C73">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="74" spans="1:3">
@@ -115301,7 +115301,7 @@
         <v>8168</v>
       </c>
       <c r="C74">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="75" spans="1:3">
@@ -115345,7 +115345,7 @@
         <v>8164</v>
       </c>
       <c r="C78">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="79" spans="1:3">
@@ -115367,7 +115367,7 @@
         <v>8162</v>
       </c>
       <c r="C80">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="81" spans="1:3">
@@ -115400,7 +115400,7 @@
         <v>8159</v>
       </c>
       <c r="C83">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="84" spans="1:3">
@@ -115411,7 +115411,7 @@
         <v>8158</v>
       </c>
       <c r="C84">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="85" spans="1:3">
@@ -115433,7 +115433,7 @@
         <v>8156</v>
       </c>
       <c r="C86">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="87" spans="1:3">
@@ -115466,7 +115466,7 @@
         <v>8153</v>
       </c>
       <c r="C89">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="90" spans="1:3">
@@ -115477,7 +115477,7 @@
         <v>8152</v>
       </c>
       <c r="C90">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -115521,7 +115521,7 @@
         <v>8148</v>
       </c>
       <c r="C94">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="95" spans="1:3">
@@ -115532,7 +115532,7 @@
         <v>8147</v>
       </c>
       <c r="C95">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="96" spans="1:3">
@@ -115543,7 +115543,7 @@
         <v>8146</v>
       </c>
       <c r="C96">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="97" spans="1:3">
@@ -115554,7 +115554,7 @@
         <v>8145</v>
       </c>
       <c r="C97">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="98" spans="1:3">
@@ -115609,7 +115609,7 @@
         <v>8140</v>
       </c>
       <c r="C102">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="103" spans="1:3">
@@ -115631,7 +115631,7 @@
         <v>8138</v>
       </c>
       <c r="C104">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105" spans="1:3">
@@ -115653,7 +115653,7 @@
         <v>8136</v>
       </c>
       <c r="C106">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="107" spans="1:3">
@@ -115686,7 +115686,7 @@
         <v>8133</v>
       </c>
       <c r="C109">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="110" spans="1:3">
@@ -115708,7 +115708,7 @@
         <v>8131</v>
       </c>
       <c r="C111">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="112" spans="1:3">
@@ -115719,7 +115719,7 @@
         <v>8130</v>
       </c>
       <c r="C112">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="113" spans="1:3">
@@ -115752,7 +115752,7 @@
         <v>8127</v>
       </c>
       <c r="C115">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="116" spans="1:3">
@@ -115774,7 +115774,7 @@
         <v>8125</v>
       </c>
       <c r="C117">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="118" spans="1:3">
@@ -115785,7 +115785,7 @@
         <v>8124</v>
       </c>
       <c r="C118">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="119" spans="1:3">
@@ -115818,7 +115818,7 @@
         <v>8121</v>
       </c>
       <c r="C121">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="122" spans="1:3">
@@ -115851,7 +115851,7 @@
         <v>8118</v>
       </c>
       <c r="C124">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="125" spans="1:3">
@@ -115873,7 +115873,7 @@
         <v>8116</v>
       </c>
       <c r="C126">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="127" spans="1:3">
@@ -115906,7 +115906,7 @@
         <v>8113</v>
       </c>
       <c r="C129">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="130" spans="1:3">
@@ -115917,7 +115917,7 @@
         <v>8112</v>
       </c>
       <c r="C130">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="131" spans="1:3">
@@ -115928,7 +115928,7 @@
         <v>8111</v>
       </c>
       <c r="C131">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="132" spans="1:3">
@@ -115939,7 +115939,7 @@
         <v>8110</v>
       </c>
       <c r="C132">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="133" spans="1:3">
@@ -115961,7 +115961,7 @@
         <v>8108</v>
       </c>
       <c r="C134">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="135" spans="1:3">
@@ -115983,7 +115983,7 @@
         <v>8106</v>
       </c>
       <c r="C136">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="137" spans="1:3">
@@ -116005,7 +116005,7 @@
         <v>8104</v>
       </c>
       <c r="C138">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="139" spans="1:3">
@@ -116027,7 +116027,7 @@
         <v>8102</v>
       </c>
       <c r="C140">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="141" spans="1:3">
@@ -116049,7 +116049,7 @@
         <v>8100</v>
       </c>
       <c r="C142">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="143" spans="1:3">
@@ -116060,7 +116060,7 @@
         <v>8099</v>
       </c>
       <c r="C143">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="144" spans="1:3">
@@ -116071,7 +116071,7 @@
         <v>8098</v>
       </c>
       <c r="C144">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="145" spans="1:3">
@@ -116082,7 +116082,7 @@
         <v>8097</v>
       </c>
       <c r="C145">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="146" spans="1:3">
@@ -116093,7 +116093,7 @@
         <v>8096</v>
       </c>
       <c r="C146">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="147" spans="1:3">
@@ -116115,7 +116115,7 @@
         <v>8094</v>
       </c>
       <c r="C148">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="149" spans="1:3">
@@ -116126,7 +116126,7 @@
         <v>8093</v>
       </c>
       <c r="C149">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="150" spans="1:3">
@@ -116137,7 +116137,7 @@
         <v>8092</v>
       </c>
       <c r="C150">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="151" spans="1:3">
@@ -116159,7 +116159,7 @@
         <v>8090</v>
       </c>
       <c r="C152">
-        <v>16</v>
+        <v>5</v>
       </c>
     </row>
     <row r="153" spans="1:3">
@@ -116203,7 +116203,7 @@
         <v>8086</v>
       </c>
       <c r="C156">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="157" spans="1:3">
@@ -116225,7 +116225,7 @@
         <v>8084</v>
       </c>
       <c r="C158">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="159" spans="1:3">
@@ -116236,7 +116236,7 @@
         <v>8083</v>
       </c>
       <c r="C159">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="160" spans="1:3">
@@ -116247,7 +116247,7 @@
         <v>8082</v>
       </c>
       <c r="C160">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="161" spans="1:3">
@@ -116291,7 +116291,7 @@
         <v>8078</v>
       </c>
       <c r="C164">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="165" spans="1:3">
@@ -116313,7 +116313,7 @@
         <v>8076</v>
       </c>
       <c r="C166">
-        <v>22</v>
+        <v>12</v>
       </c>
     </row>
     <row r="167" spans="1:3">
@@ -116357,7 +116357,7 @@
         <v>8072</v>
       </c>
       <c r="C170">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="171" spans="1:3">
@@ -116368,7 +116368,7 @@
         <v>8071</v>
       </c>
       <c r="C171">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="172" spans="1:3">
@@ -116379,7 +116379,7 @@
         <v>8069</v>
       </c>
       <c r="C172">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -116528,16 +116528,16 @@
         <v>8269</v>
       </c>
       <c r="D6" s="14">
-        <v>1318</v>
+        <v>1003</v>
       </c>
       <c r="E6" s="13" t="s">
+        <v>8271</v>
+      </c>
+      <c r="F6" s="14">
+        <v>5</v>
+      </c>
+      <c r="G6" s="15" t="s">
         <v>8270</v>
-      </c>
-      <c r="F6" s="14">
-        <v>6</v>
-      </c>
-      <c r="G6" s="15" t="s">
-        <v>8271</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="17.25" thickTop="1"/>

</xml_diff>

<commit_message>
fixed "RMSD Loss" term in figure 3 + fixed typo in Supplementary Data S1 for MobyWat set criterion
RMSD Loss -> (Capped) Displacement Loss
3A -> 3.5A (typo)
</commit_message>
<xml_diff>
--- a/SI/Supplementary Data S1/ncryst.xlsx
+++ b/SI/Supplementary Data S1/ncryst.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\GitHub\WatGNN_SI\SI\Supplementary Data S1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2B2B824-6E82-4D39-9DCC-C0A72EE1C704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{442E8EB0-F409-470A-A919-B81E5A347BAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16680" yWindow="2655" windowWidth="18060" windowHeight="11295" firstSheet="4" activeTab="6" xr2:uid="{EE483F5B-5A14-4BEB-82EA-32D6D02872BB}"/>
+    <workbookView xWindow="19785" yWindow="1785" windowWidth="18060" windowHeight="11295" firstSheet="4" activeTab="6" xr2:uid="{EE483F5B-5A14-4BEB-82EA-32D6D02872BB}"/>
   </bookViews>
   <sheets>
     <sheet name="ncryst_WatGNN_train" sheetId="2" r:id="rId1"/>
@@ -24907,15 +24907,15 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>B-factor &lt;40 Å² ref. water within 3 Å of both receptor and ligand atoms</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>7.6±5.2</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>2–16</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B-factor &lt;40 Å² ref. water within 3.5 Å of both receptor and ligand atoms</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -116698,19 +116698,19 @@
         <v>5</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>8278</v>
+        <v>8280</v>
       </c>
       <c r="D7" s="14">
         <v>38</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>8279</v>
+        <v>8278</v>
       </c>
       <c r="F7" s="14">
         <v>6</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>8280</v>
+        <v>8279</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="17.25" thickTop="1"/>

</xml_diff>